<commit_message>
events: add various events for siebnen
</commit_message>
<xml_diff>
--- a/data/events.xlsx
+++ b/data/events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sintioch-my.sharepoint.com/personal/philipp_bruhin_sintio_ch/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="11_F31306012C387D6A2061021EB8528899A12C2C28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86C3C467-4C1E-4DF3-B4C3-9817AA3F9E2E}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="11_F31306012C387D6A2061021EB8528899A12C2C28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DED45030-4924-4F28-BEC0-C3A1058B83E4}"/>
   <bookViews>
     <workbookView xWindow="-28898" yWindow="-4478" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="39">
   <si>
     <t>start</t>
   </si>
@@ -79,9 +79,6 @@
     <t>https://xn--siebnermrt-x5a.ch/</t>
   </si>
   <si>
-    <t>im Dorf</t>
-  </si>
-  <si>
     <t>Marktkommission Siebnen</t>
   </si>
   <si>
@@ -110,6 +107,36 @@
   </si>
   <si>
     <t>ab 19:00 Uhr</t>
+  </si>
+  <si>
+    <t>Musikanten-Höck</t>
+  </si>
+  <si>
+    <t>Restaurant Gusöteli</t>
+  </si>
+  <si>
+    <t>Ernst Ostertag</t>
+  </si>
+  <si>
+    <t>Ein gemütlicher Musiknachmittag - zum mitspielen, tanzen und zuhören. Jeden dritten Donnerstag im Monat.</t>
+  </si>
+  <si>
+    <t>https://www.ostertagmusik.com/</t>
+  </si>
+  <si>
+    <t>https://www.siebner-fasnacht.ch/</t>
+  </si>
+  <si>
+    <t>Einschellen 2026</t>
+  </si>
+  <si>
+    <t>Dorf Siebnen</t>
+  </si>
+  <si>
+    <t>Los geht es ab 19:37 Uhr.</t>
+  </si>
+  <si>
+    <t>Dachorganisation Siebner Fasnach</t>
   </si>
 </sst>
 </file>
@@ -184,13 +211,13 @@
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -215,16 +242,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}" name="Table1" displayName="Table1" ref="A1:G6" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:G6" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}" name="Table1" displayName="Table1" ref="A1:G16" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:G16" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{AC1863B4-E7E6-450C-B42D-02C152549B53}" name="start" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{B687C935-5EAB-43E5-AC23-2AEE75E32F94}" name="end" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{7EED7B55-DCA2-48F3-80EF-D977C6C62484}" name="name" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{553A63A7-14F1-46D5-B4AE-504CDA399DDE}" name="description" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{6C0DC369-4C2B-4FC3-B790-830F7C50DFEB}" name="location" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{E0A5A1F9-C4D2-4895-9EB9-9FBCD5E1303A}" name="organizer" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{E1D0A691-8F43-436E-A4C1-C7A138BC34A5}" name="url" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{AC1863B4-E7E6-450C-B42D-02C152549B53}" name="start" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{B687C935-5EAB-43E5-AC23-2AEE75E32F94}" name="end" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{7EED7B55-DCA2-48F3-80EF-D977C6C62484}" name="name" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{553A63A7-14F1-46D5-B4AE-504CDA399DDE}" name="description" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{6C0DC369-4C2B-4FC3-B790-830F7C50DFEB}" name="location" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{E0A5A1F9-C4D2-4895-9EB9-9FBCD5E1303A}" name="organizer" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{E1D0A691-8F43-436E-A4C1-C7A138BC34A5}" name="url" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -552,14 +579,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="10.125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.5" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="59.25" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.75" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="44" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9" style="1"/>
   </cols>
@@ -589,121 +616,318 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
-        <v>46127</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>46028</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <v>46129</v>
-      </c>
-      <c r="B3" s="3">
-        <v>46130</v>
+        <v>46123</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
-        <v>46284</v>
+        <v>46127</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <v>46292</v>
+        <v>46129</v>
       </c>
       <c r="B5" s="3">
-        <v>46294</v>
+        <v>46130</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
+        <v>46163</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>46191</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>46219</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
+        <v>46254</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>46282</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>46284</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>46292</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46294</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>46310</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>46345</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
         <v>46359</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{C5235A01-AD86-4881-94BB-4DB56A8B0429}"/>
-    <hyperlink ref="G3" r:id="rId2" xr:uid="{117B3DE2-8D42-40B0-AAB0-CEA6866D784F}"/>
-    <hyperlink ref="G5" r:id="rId3" xr:uid="{9896CDBD-F6C1-4826-962B-B144E084E4A9}"/>
-    <hyperlink ref="G6" r:id="rId4" xr:uid="{76233139-11D1-4AC8-8C9F-A261DF3FBAB8}"/>
-    <hyperlink ref="G4" r:id="rId5" xr:uid="{C862A952-4001-41B9-923A-B16E51BA1C52}"/>
+    <hyperlink ref="G4" r:id="rId1" xr:uid="{C5235A01-AD86-4881-94BB-4DB56A8B0429}"/>
+    <hyperlink ref="G5" r:id="rId2" xr:uid="{117B3DE2-8D42-40B0-AAB0-CEA6866D784F}"/>
+    <hyperlink ref="G12" r:id="rId3" xr:uid="{9896CDBD-F6C1-4826-962B-B144E084E4A9}"/>
+    <hyperlink ref="G16" r:id="rId4" xr:uid="{76233139-11D1-4AC8-8C9F-A261DF3FBAB8}"/>
+    <hyperlink ref="G11" r:id="rId5" xr:uid="{C862A952-4001-41B9-923A-B16E51BA1C52}"/>
+    <hyperlink ref="G6" r:id="rId6" xr:uid="{660747D9-377B-47FC-A7D5-B7D35D990DBD}"/>
+    <hyperlink ref="G3" r:id="rId7" xr:uid="{5A36D3D6-51C9-47DE-BDE4-DEA5C45E3F44}"/>
+    <hyperlink ref="G7" r:id="rId8" xr:uid="{851A95D2-10CF-4306-B429-0FB267FEA1A5}"/>
+    <hyperlink ref="G8" r:id="rId9" xr:uid="{178A6F0E-39C5-41A9-B60B-36426E389A8C}"/>
+    <hyperlink ref="G9" r:id="rId10" xr:uid="{93D295A3-0420-4B25-9334-8F673699464F}"/>
+    <hyperlink ref="G10" r:id="rId11" xr:uid="{727E350B-787A-4EEF-89D5-D64AA2A9B90C}"/>
+    <hyperlink ref="G13" r:id="rId12" xr:uid="{BA517086-7632-41F8-AE54-49A35A96F980}"/>
+    <hyperlink ref="G15" r:id="rId13" xr:uid="{FFB772E1-4081-43E7-B964-E8EB13D63EA6}"/>
+    <hyperlink ref="G2" r:id="rId14" xr:uid="{C24412FA-B74F-4FEA-A2F1-4667B0DA0451}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: add siebnen page and rearange content
</commit_message>
<xml_diff>
--- a/data/events.xlsx
+++ b/data/events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sintioch-my.sharepoint.com/personal/philipp_bruhin_sintio_ch/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/philippbruhin/Documents/repos/7eichen-website/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="11_F31306012C387D6A2061021EB8528899A12C2C28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DED45030-4924-4F28-BEC0-C3A1058B83E4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D032FBEA-C0B4-BF40-A17D-9E3948E85555}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28898" yWindow="-4478" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Termine" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="44">
   <si>
     <t>start</t>
   </si>
@@ -137,6 +137,21 @@
   </si>
   <si>
     <t>Dachorganisation Siebner Fasnach</t>
+  </si>
+  <si>
+    <t>Street Food Park Festival</t>
+  </si>
+  <si>
+    <t>30 Food Trucks und Food Stände</t>
+  </si>
+  <si>
+    <t>Chilbiplatz Siebnen</t>
+  </si>
+  <si>
+    <t>Alta Vista Events</t>
+  </si>
+  <si>
+    <t>https://www.streetfood-park.com/</t>
   </si>
 </sst>
 </file>
@@ -242,8 +257,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}" name="Table1" displayName="Table1" ref="A1:G16" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:G16" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}" name="Table1" displayName="Table1" ref="A1:G17" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:G17" xr:uid="{3627BE0B-73F9-4A9A-A395-BA0A746F30CB}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{AC1863B4-E7E6-450C-B42D-02C152549B53}" name="start" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{B687C935-5EAB-43E5-AC23-2AEE75E32F94}" name="end" dataDxfId="5"/>
@@ -579,19 +594,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="59.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="59.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="44" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -614,7 +629,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>46028</v>
       </c>
@@ -635,7 +650,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>46123</v>
       </c>
@@ -655,7 +670,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>46127</v>
       </c>
@@ -675,7 +690,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>46129</v>
       </c>
@@ -698,7 +713,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>46163</v>
       </c>
@@ -719,7 +734,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>46191</v>
       </c>
@@ -740,30 +755,32 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
+        <v>46199</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46201</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
         <v>46219</v>
-      </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
-        <v>46254</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="1" t="s">
@@ -782,9 +799,9 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>46282</v>
+        <v>46254</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="1" t="s">
@@ -803,108 +820,129 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
+        <v>46282</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
         <v>46284</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
+    <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
         <v>46292</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B13" s="3">
         <v>46294</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+    <row r="14" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
         <v>46310</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="1" t="s">
+      <c r="B14" s="3"/>
+      <c r="C14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G14" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+    <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
         <v>46345</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="1" t="s">
+      <c r="B16" s="3"/>
+      <c r="C16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+    <row r="17" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
         <v>46359</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>22</v>
       </c>
     </row>
@@ -912,22 +950,23 @@
   <hyperlinks>
     <hyperlink ref="G4" r:id="rId1" xr:uid="{C5235A01-AD86-4881-94BB-4DB56A8B0429}"/>
     <hyperlink ref="G5" r:id="rId2" xr:uid="{117B3DE2-8D42-40B0-AAB0-CEA6866D784F}"/>
-    <hyperlink ref="G12" r:id="rId3" xr:uid="{9896CDBD-F6C1-4826-962B-B144E084E4A9}"/>
-    <hyperlink ref="G16" r:id="rId4" xr:uid="{76233139-11D1-4AC8-8C9F-A261DF3FBAB8}"/>
-    <hyperlink ref="G11" r:id="rId5" xr:uid="{C862A952-4001-41B9-923A-B16E51BA1C52}"/>
+    <hyperlink ref="G13" r:id="rId3" xr:uid="{9896CDBD-F6C1-4826-962B-B144E084E4A9}"/>
+    <hyperlink ref="G17" r:id="rId4" xr:uid="{76233139-11D1-4AC8-8C9F-A261DF3FBAB8}"/>
+    <hyperlink ref="G12" r:id="rId5" xr:uid="{C862A952-4001-41B9-923A-B16E51BA1C52}"/>
     <hyperlink ref="G6" r:id="rId6" xr:uid="{660747D9-377B-47FC-A7D5-B7D35D990DBD}"/>
     <hyperlink ref="G3" r:id="rId7" xr:uid="{5A36D3D6-51C9-47DE-BDE4-DEA5C45E3F44}"/>
     <hyperlink ref="G7" r:id="rId8" xr:uid="{851A95D2-10CF-4306-B429-0FB267FEA1A5}"/>
-    <hyperlink ref="G8" r:id="rId9" xr:uid="{178A6F0E-39C5-41A9-B60B-36426E389A8C}"/>
-    <hyperlink ref="G9" r:id="rId10" xr:uid="{93D295A3-0420-4B25-9334-8F673699464F}"/>
-    <hyperlink ref="G10" r:id="rId11" xr:uid="{727E350B-787A-4EEF-89D5-D64AA2A9B90C}"/>
-    <hyperlink ref="G13" r:id="rId12" xr:uid="{BA517086-7632-41F8-AE54-49A35A96F980}"/>
-    <hyperlink ref="G15" r:id="rId13" xr:uid="{FFB772E1-4081-43E7-B964-E8EB13D63EA6}"/>
+    <hyperlink ref="G9" r:id="rId9" xr:uid="{178A6F0E-39C5-41A9-B60B-36426E389A8C}"/>
+    <hyperlink ref="G10" r:id="rId10" xr:uid="{93D295A3-0420-4B25-9334-8F673699464F}"/>
+    <hyperlink ref="G11" r:id="rId11" xr:uid="{727E350B-787A-4EEF-89D5-D64AA2A9B90C}"/>
+    <hyperlink ref="G14" r:id="rId12" xr:uid="{BA517086-7632-41F8-AE54-49A35A96F980}"/>
+    <hyperlink ref="G16" r:id="rId13" xr:uid="{FFB772E1-4081-43E7-B964-E8EB13D63EA6}"/>
     <hyperlink ref="G2" r:id="rId14" xr:uid="{C24412FA-B74F-4FEA-A2F1-4667B0DA0451}"/>
+    <hyperlink ref="G8" r:id="rId15" xr:uid="{1D45EB05-0B76-8E48-88B4-9A7BEA5E81C7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>